<commit_message>
Restructure backend-excel codebase into modular, object-oriented services (Excel, Auth, Bet, Match services)
</commit_message>
<xml_diff>
--- a/backend-excel/data/accounts.xlsx
+++ b/backend-excel/data/accounts.xlsx
@@ -424,7 +424,7 @@
         <v>admin</v>
       </c>
       <c r="C2" t="str">
-        <v>$2a$10$6HspttK4awNpNyaz0uVHpeaoN9cFQdoImjH9518tbhg09zY/Lc1UO</v>
+        <v>$2a$10$TbKN0dEKURg14kYcVgXiYu2pTkxakk4HBie.umFrWdAgdiZWFKbMi</v>
       </c>
       <c r="D2" t="str">
         <v>Administrator</v>
@@ -441,7 +441,7 @@
         <v>lctran</v>
       </c>
       <c r="C3" t="str">
-        <v>$2a$10$uUaitW12.mQanftv0aN6ieWbceceQ12qJqjt9t2oOiPGgebWHc3Z.</v>
+        <v>$2a$10$.aq9vYRe8P59YMXHabrROuSHvgyXhxUABop.67XnSKBNsIMVNDPIy</v>
       </c>
       <c r="D3" t="str">
         <v>Tran Chanh Luan</v>
@@ -458,7 +458,7 @@
         <v>cam</v>
       </c>
       <c r="C4" t="str">
-        <v>$2a$10$7KH/Jm9WzgTaS9W0J1PVqOi0suLvlkSvdxG3f0P6rofSPszr9bEV6</v>
+        <v>$2a$10$cegUMS9..lnU2gFKgmDKPuYzCeGOBLWeSiD.eM3GN.PzIC5hP8R8K</v>
       </c>
       <c r="D4" t="str">
         <v>Nguyễn Thị Cam</v>
@@ -475,7 +475,7 @@
         <v>test</v>
       </c>
       <c r="C5" t="str">
-        <v>$2a$10$7KH/Jm9WzgTaS9W0J1PVqOi0suLvlkSvdxG3f0P6rofSPszr9bEV6</v>
+        <v>$2a$10$Be5q9ZuOnHAMYT8Z3OAi/.8xtpIcuWPGe610ClsBNzACiNRWZrqfG</v>
       </c>
       <c r="D5" t="str">
         <v>test</v>

</xml_diff>

<commit_message>
fix: resolve frozen live match status by correcting sync state progression and merging logic
</commit_message>
<xml_diff>
--- a/backend-excel/data/accounts.xlsx
+++ b/backend-excel/data/accounts.xlsx
@@ -424,7 +424,7 @@
         <v>admin</v>
       </c>
       <c r="C2" t="str">
-        <v>$2a$10$9HpgCwgN3eI2m3PekH.Ztu9qot1hsC1kS8sFjBQdLkfktvUnBTsty</v>
+        <v>$2a$10$9qbCwNF3M37kQGO2Q7A.meIpOdyZDf/AQB/tr6JI0efGsSx62rvwi</v>
       </c>
       <c r="D2" t="str">
         <v>Administrator</v>
@@ -441,7 +441,7 @@
         <v>lctran</v>
       </c>
       <c r="C3" t="str">
-        <v>$2a$10$D4VO3B7eplyFuAy7dth2aOO2H/a21VXEr2EhUNnVVzLxfzfFQk6k.</v>
+        <v>$2a$10$7102X88SMhaXjgvcS4uPNeKLDaB.BEuvYREwr0QMAlh7Ap1MQumdC</v>
       </c>
       <c r="D3" t="str">
         <v>Tran Chanh Luan</v>
@@ -458,7 +458,7 @@
         <v>cam</v>
       </c>
       <c r="C4" t="str">
-        <v>$2a$10$IPt3KMUCnPt9zXMx9yZPp.8U.jOC1gMcrWbrDdNOlVQqmBp6xDhXa</v>
+        <v>$2a$10$a2Nn2dlp6NDHGujxm0iKS.mcuD9CTI7zBszGftqYo8305rapG6ejO</v>
       </c>
       <c r="D4" t="str">
         <v>Nguyễn Thị Cam</v>
@@ -475,7 +475,7 @@
         <v>test</v>
       </c>
       <c r="C5" t="str">
-        <v>$2a$10$BApe2cDr5pl6tBiZzcD9LOLGVh6gcaXd8tdFgUg/S6CNs52UmHvMC</v>
+        <v>$2a$10$54LjT1jWokPyd5jdxHbJVOsB8NWv9h8BcGXu6mmaQcyn0KM6Hq1mS</v>
       </c>
       <c r="D5" t="str">
         <v>test</v>

</xml_diff>